<commit_message>
Vermieter-Toolkit: Strategie, Modul Wohnungsrückgabe und Korrekturen
- STRATEGIE.md: Marktanalyse, Bewertung der fuenf Module, 20 Kandidaten
  fuer die sechste Funktion mit Score, Architektur, Preis und Pruefbericht
- Neues Modul «Wohnungsrückgabe: Schaden & Kaution»: Mieteranteil nach
  Lebensdauer, Kautionsabrechnung, Freigabe fuer die Bank; 11 Prueffaelle
- Nebenkosten: Kontrolle meldet jetzt Mietende vor Mietbeginn und
  Kostenarten mit Schluessel-Total 0 (vorher stillschweigend beim
  Eigentuemer); neue Pruefstrecke mit 23 Faellen
- Website: ein Angebot «Vermieter-Ordner Schweiz», Einfuehrungspreis
  CHF 39 bis 31.12.2026, danach CHF 49, 14 Tage Geld-zurueck

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VzYvY4qj4r3T84VcSe7CSt
</commit_message>
<xml_diff>
--- a/money-agent/products/nebenkosten-ch/Nebenkostenabrechnung-CH-Beispiel.xlsx
+++ b/money-agent/products/nebenkosten-ch/Nebenkostenabrechnung-CH-Beispiel.xlsx
@@ -12038,7 +12038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12147,25 +12147,47 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Mietende vor Mietbeginn</t>
+        </is>
+      </c>
+      <c r="B12" s="13">
+        <f>SUMPRODUCT((Mieter!C5:C44&lt;&gt;"")*(Mieter!D5:D44&lt;&gt;"")*(Mieter!E5:E44&lt;&gt;"")*(Mieter!E5:E44&lt;Mieter!D5:D44))</f>
+        <v/>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Kostenarten mit Schlüssel-Total 0 (z.B. keine Anteile erfasst)</t>
+        </is>
+      </c>
+      <c r="B13" s="13">
+        <f>SUMPRODUCT((Kosten!B5:B29&lt;&gt;"")*(Kosten!C5:C29&lt;&gt;"")*(Kosten!E5:E29=0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B13" s="22">
-        <f>IF(AND(B7=0,B8=1000,B9=0,B10=0,B11=0),"OK","Bitte prüfen")</f>
+      <c r="B15" s="22">
+        <f>IF(AND(B7=0,B8=1000,B9=0,B10=0,B11=0,B12=0,B13=0),"OK","Bitte prüfen")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <conditionalFormatting sqref="B13">
+  <conditionalFormatting sqref="B15">
     <cfRule type="expression" priority="1" dxfId="1">
-      <formula>B13="OK"</formula>
+      <formula>B15="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>B13&lt;&gt;"OK"</formula>
+      <formula>B15&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>